<commit_message>
nmv 22 02 2026
</commit_message>
<xml_diff>
--- a/TS Jatai Working/Padam Input Templates/TS 6.5 Padam Input Template.xlsx
+++ b/TS Jatai Working/Padam Input Templates/TS 6.5 Padam Input Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ALL IMP DATA\GitHub\texts\TS Jatai Working\Padam Input Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDE9216D-B0CF-4F8A-9726-2C24A8051455}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7236A30A-2EE3-4DEA-9B49-1F52572C41B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5547" uniqueCount="1232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5547" uniqueCount="1233">
   <si>
     <t>Passage</t>
   </si>
@@ -3788,6 +3788,9 @@
   </si>
   <si>
     <t xml:space="preserve">RuqtU ityRuqtU </t>
+  </si>
+  <si>
+    <t xml:space="preserve">uqpAq(gm)qSu </t>
   </si>
 </sst>
 </file>
@@ -54849,8 +54852,8 @@
         <f t="shared" si="71"/>
         <v>234</v>
       </c>
-      <c r="N1495" s="45" t="s">
-        <v>724</v>
+      <c r="N1495" s="46" t="s">
+        <v>1232</v>
       </c>
       <c r="O1495" s="8" t="s">
         <v>62</v>

</xml_diff>

<commit_message>
nmv 28 02 2026
</commit_message>
<xml_diff>
--- a/TS Jatai Working/Padam Input Templates/TS 6.5 Padam Input Template.xlsx
+++ b/TS Jatai Working/Padam Input Templates/TS 6.5 Padam Input Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ALL IMP DATA\GitHub\texts\TS Jatai Working\Padam Input Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7236A30A-2EE3-4DEA-9B49-1F52572C41B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0243FCB-3272-49E0-94AF-F0F3EC4E2C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3547,9 +3547,6 @@
   </si>
   <si>
     <t xml:space="preserve">Aqdiqtyaqgraqha ityA#ditya - graqhaH </t>
-  </si>
-  <si>
-    <t xml:space="preserve">uqpAq(gm)qSumityu#pa - aqSum </t>
   </si>
   <si>
     <t xml:space="preserve">viqgRuqhNAtIti# vi - gRuqhNAti# </t>
@@ -3791,6 +3788,9 @@
   </si>
   <si>
     <t xml:space="preserve">uqpAq(gm)qSu </t>
+  </si>
+  <si>
+    <t xml:space="preserve">uqpAq(gm)qSumityu#pa - aq(gm)qSum </t>
   </si>
 </sst>
 </file>
@@ -5692,7 +5692,7 @@
         <v>76</v>
       </c>
       <c r="T17" s="17" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="U17" s="17"/>
       <c r="V17" s="45"/>
@@ -9973,7 +9973,7 @@
         <v>70</v>
       </c>
       <c r="T135" s="8" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="U135" s="8"/>
       <c r="V135" s="45"/>
@@ -10510,7 +10510,7 @@
         <v>76</v>
       </c>
       <c r="T151" s="8" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="U151" s="8"/>
       <c r="V151" s="45" t="s">
@@ -10986,7 +10986,7 @@
       <c r="S165" s="8"/>
       <c r="T165" s="8"/>
       <c r="U165" s="8" t="s">
-        <v>1214</v>
+        <v>1213</v>
       </c>
       <c r="V165" s="45" t="s">
         <v>971</v>
@@ -12110,7 +12110,7 @@
         <v>73</v>
       </c>
       <c r="T199" s="8" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="U199" s="8"/>
       <c r="V199" s="45"/>
@@ -13843,7 +13843,7 @@
       <c r="S250" s="8"/>
       <c r="T250" s="8"/>
       <c r="U250" s="8" t="s">
-        <v>1214</v>
+        <v>1213</v>
       </c>
       <c r="V250" s="45"/>
     </row>
@@ -15067,7 +15067,7 @@
         <v>53</v>
       </c>
       <c r="N287" s="45" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="O287" s="8" t="s">
         <v>62</v>
@@ -19319,7 +19319,7 @@
         <v>41</v>
       </c>
       <c r="N414" s="46" t="s">
-        <v>1224</v>
+        <v>1223</v>
       </c>
       <c r="O414" s="7" t="s">
         <v>64</v>
@@ -19503,7 +19503,7 @@
       <c r="T419" s="8"/>
       <c r="U419" s="8"/>
       <c r="V419" s="46" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="420" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
@@ -19838,7 +19838,7 @@
     </row>
     <row r="430" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A430" s="60" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="B430" s="55"/>
       <c r="C430" s="55"/>
@@ -20598,7 +20598,7 @@
         <v>76</v>
       </c>
       <c r="T451" s="8" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="U451" s="8"/>
       <c r="V451" s="45"/>
@@ -20814,7 +20814,7 @@
     </row>
     <row r="458" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A458" s="60" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="D458" s="24"/>
       <c r="I458" s="48" t="s">
@@ -21167,7 +21167,7 @@
         <v>95</v>
       </c>
       <c r="N468" s="46" t="s">
-        <v>1228</v>
+        <v>1227</v>
       </c>
       <c r="O468" s="8" t="s">
         <v>62</v>
@@ -21252,7 +21252,7 @@
     </row>
     <row r="471" spans="1:22" s="5" customFormat="1" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A471" s="8" t="s">
-        <v>1219</v>
+        <v>1218</v>
       </c>
       <c r="D471" s="24"/>
       <c r="H471" s="50" t="s">
@@ -21387,7 +21387,7 @@
         <v>76</v>
       </c>
       <c r="T474" s="8" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="U474" s="8"/>
       <c r="V474" s="45"/>
@@ -22063,7 +22063,7 @@
         <v>76</v>
       </c>
       <c r="T494" s="8" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="U494" s="8"/>
       <c r="V494" s="45"/>
@@ -26004,7 +26004,7 @@
         <v>53</v>
       </c>
       <c r="N610" s="46" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="O610" s="7"/>
       <c r="P610" s="8"/>
@@ -27915,7 +27915,7 @@
     </row>
     <row r="668" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A668" s="61" t="s">
-        <v>1220</v>
+        <v>1219</v>
       </c>
       <c r="H668" s="50" t="s">
         <v>89</v>
@@ -28899,7 +28899,7 @@
     </row>
     <row r="699" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A699" s="62" t="s">
-        <v>1221</v>
+        <v>1220</v>
       </c>
       <c r="I699" s="48" t="s">
         <v>35</v>
@@ -35866,7 +35866,7 @@
     </row>
     <row r="917" spans="1:22" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A917" s="63" t="s">
-        <v>1222</v>
+        <v>1221</v>
       </c>
       <c r="H917" s="50" t="s">
         <v>92</v>
@@ -35900,7 +35900,7 @@
         <v>76</v>
       </c>
       <c r="T917" s="8" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="U917" s="8"/>
       <c r="V917" s="45"/>
@@ -36752,7 +36752,7 @@
         <v>81</v>
       </c>
       <c r="T942" s="8" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="U942" s="8"/>
       <c r="V942" s="45"/>
@@ -43134,7 +43134,7 @@
         <v>81</v>
       </c>
       <c r="T1140" s="8" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="U1140" s="8"/>
       <c r="V1140" s="45"/>
@@ -43659,7 +43659,7 @@
         <v>81</v>
       </c>
       <c r="T1156" s="8" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
       <c r="V1156" s="45"/>
     </row>
@@ -47062,7 +47062,7 @@
         <v>1</v>
       </c>
       <c r="N1262" s="46" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="O1262" s="8" t="s">
         <v>62</v>
@@ -47915,7 +47915,7 @@
         <v>27</v>
       </c>
       <c r="N1288" s="46" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="O1288" s="8" t="s">
         <v>62</v>
@@ -47927,7 +47927,7 @@
       <c r="T1288" s="8"/>
       <c r="U1288" s="8"/>
       <c r="V1288" s="46" t="s">
-        <v>1225</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="1289" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -51681,7 +51681,7 @@
       <c r="T1400" s="8"/>
       <c r="U1400" s="8"/>
       <c r="V1400" s="46" t="s">
-        <v>1229</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="1401" spans="3:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -52010,7 +52010,7 @@
         <v>149</v>
       </c>
       <c r="N1410" s="46" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
       <c r="O1410" s="8" t="s">
         <v>62</v>
@@ -52385,7 +52385,7 @@
         <v>160</v>
       </c>
       <c r="N1421" s="68" t="s">
-        <v>1223</v>
+        <v>1222</v>
       </c>
       <c r="O1421" s="7"/>
       <c r="P1421" s="8"/>
@@ -54853,7 +54853,7 @@
         <v>234</v>
       </c>
       <c r="N1495" s="46" t="s">
-        <v>1232</v>
+        <v>1231</v>
       </c>
       <c r="O1495" s="8" t="s">
         <v>62</v>
@@ -55333,7 +55333,7 @@
         <v>248</v>
       </c>
       <c r="N1509" s="46" t="s">
-        <v>1230</v>
+        <v>1229</v>
       </c>
       <c r="O1509" s="8" t="s">
         <v>62</v>
@@ -60598,7 +60598,7 @@
         <v>76</v>
       </c>
       <c r="T1694" s="8" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="V1694" s="45"/>
     </row>
@@ -62512,10 +62512,10 @@
         <v>63</v>
       </c>
       <c r="S1769" s="8" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="T1769" s="8" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
       <c r="V1769" s="46" t="s">
         <v>1165</v>
@@ -63195,8 +63195,8 @@
       <c r="O1795" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="V1795" s="45" t="s">
-        <v>1173</v>
+      <c r="V1795" s="46" t="s">
+        <v>1232</v>
       </c>
     </row>
     <row r="1796" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -63249,7 +63249,7 @@
         <v>62</v>
       </c>
       <c r="V1797" s="45" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="1798" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -63710,7 +63710,7 @@
         <v>62</v>
       </c>
       <c r="V1815" s="45" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="1816" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -63882,7 +63882,7 @@
         <v>62</v>
       </c>
       <c r="V1822" s="45" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="1823" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -64031,7 +64031,7 @@
         <v>62</v>
       </c>
       <c r="V1828" s="45" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="1829" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -64204,7 +64204,7 @@
         <v>62</v>
       </c>
       <c r="V1835" s="45" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="1836" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -64569,7 +64569,7 @@
         <v>62</v>
       </c>
       <c r="V1850" s="45" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="1851" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -64758,10 +64758,10 @@
         <v>65</v>
       </c>
       <c r="S1857" s="8" t="s">
+        <v>1206</v>
+      </c>
+      <c r="T1857" s="8" t="s">
         <v>1207</v>
-      </c>
-      <c r="T1857" s="8" t="s">
-        <v>1208</v>
       </c>
       <c r="V1857" s="45"/>
     </row>
@@ -64815,7 +64815,7 @@
         <v>62</v>
       </c>
       <c r="V1859" s="45" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="1860" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -65077,7 +65077,7 @@
         <v>101</v>
       </c>
       <c r="N1870" s="46" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="V1870" s="45"/>
     </row>
@@ -65107,7 +65107,7 @@
         <v>62</v>
       </c>
       <c r="V1871" s="45" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="1872" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -65136,7 +65136,7 @@
         <v>62</v>
       </c>
       <c r="V1872" s="45" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="1873" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -65165,7 +65165,7 @@
         <v>62</v>
       </c>
       <c r="V1873" s="45" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="1874" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -65632,7 +65632,7 @@
         <v>62</v>
       </c>
       <c r="V1891" s="45" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="1892" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -65733,7 +65733,7 @@
         <v>62</v>
       </c>
       <c r="V1895" s="45" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="1896" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -65963,7 +65963,7 @@
         <v>62</v>
       </c>
       <c r="V1904" s="45" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="1905" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -66223,7 +66223,7 @@
         <v>62</v>
       </c>
       <c r="V1914" s="45" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="1915" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -66252,7 +66252,7 @@
         <v>62</v>
       </c>
       <c r="V1915" s="45" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="1916" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -66659,7 +66659,7 @@
         <v>62</v>
       </c>
       <c r="V1931" s="45" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="1932" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -66736,7 +66736,7 @@
         <v>62</v>
       </c>
       <c r="V1934" s="45" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="1935" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -66813,7 +66813,7 @@
         <v>63</v>
       </c>
       <c r="V1937" s="45" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="1938" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -67035,7 +67035,7 @@
         <v>62</v>
       </c>
       <c r="V1946" s="45" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="1947" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -67355,7 +67355,7 @@
         <v>76</v>
       </c>
       <c r="T1959" s="8" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="V1959" s="45"/>
     </row>
@@ -67387,7 +67387,7 @@
       <c r="S1960" s="8"/>
       <c r="T1960" s="8"/>
       <c r="V1960" s="45" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="1961" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -67578,7 +67578,7 @@
         <v>76</v>
       </c>
       <c r="T1967" s="8" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="V1967" s="45" t="s">
         <v>969</v>
@@ -67901,7 +67901,7 @@
         <v>62</v>
       </c>
       <c r="V1980" s="45" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="1981" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -68080,7 +68080,7 @@
         <v>76</v>
       </c>
       <c r="T1987" s="1" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="V1987" s="45"/>
     </row>
@@ -68109,7 +68109,7 @@
         <v>62</v>
       </c>
       <c r="V1988" s="45" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="1989" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -68213,7 +68213,7 @@
         <v>76</v>
       </c>
       <c r="T1992" s="1" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="V1992" s="45"/>
     </row>
@@ -68489,7 +68489,7 @@
         <v>62</v>
       </c>
       <c r="V2003" s="45" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="2004" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -68716,7 +68716,7 @@
         <v>76</v>
       </c>
       <c r="T2012" s="1" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="V2012" s="45"/>
     </row>
@@ -68746,7 +68746,7 @@
         <v>62</v>
       </c>
       <c r="V2013" s="45" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="2014" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -68898,7 +68898,7 @@
         <v>62</v>
       </c>
       <c r="V2019" s="45" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="2020" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -68999,7 +68999,7 @@
         <v>62</v>
       </c>
       <c r="V2023" s="45" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="2024" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -69052,7 +69052,7 @@
         <v>62</v>
       </c>
       <c r="V2025" s="45" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="2026" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -69249,7 +69249,7 @@
         <v>62</v>
       </c>
       <c r="V2033" s="45" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="2034" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -69378,7 +69378,7 @@
         <v>62</v>
       </c>
       <c r="V2038" s="45" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="2039" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -69599,7 +69599,7 @@
         <v>62</v>
       </c>
       <c r="V2047" s="45" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="2048" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -69700,7 +69700,7 @@
         <v>62</v>
       </c>
       <c r="V2051" s="45" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="2052" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -69900,7 +69900,7 @@
         <v>62</v>
       </c>
       <c r="V2059" s="45" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="2060" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -69929,7 +69929,7 @@
         <v>62</v>
       </c>
       <c r="V2060" s="45" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="2061" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -70345,7 +70345,7 @@
         <v>62</v>
       </c>
       <c r="V2077" s="45" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="2078" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -70374,7 +70374,7 @@
         <v>62</v>
       </c>
       <c r="V2078" s="45" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="2079" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -70523,7 +70523,7 @@
         <v>62</v>
       </c>
       <c r="V2084" s="45" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="2085" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -70594,7 +70594,7 @@
         <v>150</v>
       </c>
       <c r="N2087" s="46" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="V2087" s="45"/>
     </row>
@@ -70722,7 +70722,7 @@
         <v>62</v>
       </c>
       <c r="V2092" s="45" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="2093" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -70847,7 +70847,7 @@
         <v>62</v>
       </c>
       <c r="V2097" s="45" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="2098" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -70963,7 +70963,7 @@
         <v>70</v>
       </c>
       <c r="T2101" s="8" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="V2101" s="45"/>
     </row>
@@ -71116,7 +71116,7 @@
         <v>62</v>
       </c>
       <c r="V2107" s="45" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="2108" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -71193,7 +71193,7 @@
         <v>62</v>
       </c>
       <c r="V2110" s="45" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="2111" spans="8:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -71246,10 +71246,10 @@
         <v>65</v>
       </c>
       <c r="S2112" s="8" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="T2112" s="8" t="s">
-        <v>1213</v>
+        <v>1212</v>
       </c>
       <c r="V2112" s="45"/>
     </row>
@@ -71327,7 +71327,7 @@
         <v>62</v>
       </c>
       <c r="V2115" s="45" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="2116" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -71479,7 +71479,7 @@
         <v>62</v>
       </c>
       <c r="V2121" s="45" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="2122" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -71655,7 +71655,7 @@
         <v>62</v>
       </c>
       <c r="V2128" s="45" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="2129" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -71924,7 +71924,7 @@
         <v>62</v>
       </c>
       <c r="V2139" s="45" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="2140" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -72025,7 +72025,7 @@
         <v>62</v>
       </c>
       <c r="V2143" s="45" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="2144" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">
@@ -72225,7 +72225,7 @@
         <v>63</v>
       </c>
       <c r="V2151" s="45" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>